<commit_message>
Corrección en base de datos de pipelines
</commit_message>
<xml_diff>
--- a/data/database/specs.xlsx
+++ b/data/database/specs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,22 +451,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>pipeline_id</t>
+          <t>config_json</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>config_json</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>updated_at</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>config_path</t>
         </is>
       </c>
     </row>
@@ -489,20 +479,14 @@
           <t>ETL Archivo</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{"variables_documento": {"leftimage": "", "rightimage": "", "centerheaderone": "", "centerheadertwo": "", "centerheaderthree": "", "leftfooter": "", "rightfooter": "", "documenttitle": "", "schoolname": "", "theauthor": ""}, "secciones_fijas": [], "secciones_dinamicas": [], "etlParams": [{"id": "header_row", "type": "text", "label": "Fila Encabezado", "value": "23", "config": {"id": "header_row", "label": "Fila Encabezado", "type": "text", "limit": 1}}, {"id": "output_name", "type": "text", "label": "Nombre Salida", "value": "simce_2025_estudiantes.xlsx", "config": {"id": "output_name", "label": "Nombre Salida", "type": "text", "limit": 1}}, {"id": "select_columns", "type": "list_text", "label": "Seleccionar Columnas", "value": ["Nombre", "RUT", "Curso", "B", "M", "O", "Puntaje", "Rend", "SIMCE", "Nota", "Logro"], "config": {"id": "select_columns", "label": "Seleccionar Columnas", "type": "list_text", "limit": 0}}, {"id": "rename_columns", "type": "list_pair", "label": "Renombrar Columnas", "value": [{"key": "B", "val": "Buenas"}, {"key": "M", "val": "Malas"}, {"key": "O", "val": "Omitidas"}], "config": {"id": "rename_columns", "label": "Renombrar Columnas", "type": "list_pair", "limit": 0, "fields": ["Original", "Final"]}}, {"id": "enrich_data", "type": "list_pair", "label": "Enriquecer Data", "value": [{"key": "Año", "val": "2025"}, {"key": "Asignatura", "val": "Lenguaje"}, {"key": "Mes", "val": "Noviembre"}, {"key": "N Prueba", "val": "5"}], "config": {"id": "enrich_data", "label": "Enriquecer Data", "type": "list_pair", "limit": 0, "fields": ["Columna", "Valor"]}}]}</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{"variables_documento": {"leftimage": "", "rightimage": "", "centerheaderone": "", "centerheadertwo": "", "centerheaderthree": "", "leftfooter": "", "rightfooter": "", "documenttitle": "", "schoolname": "", "theauthor": ""}, "secciones_fijas": [], "secciones_dinamicas": [], "etlParams": [{"id": "header_row", "type": "text", "label": "Fila Encabezado", "value": "23", "config": {"id": "header_row", "label": "Fila Encabezado", "type": "text", "limit": 1}}, {"id": "output_name", "type": "text", "label": "Nombre Salida", "value": "simce_2025_estudiantes.xlsx", "config": {"id": "output_name", "label": "Nombre Salida", "type": "text", "limit": 1}}, {"id": "select_columns", "type": "list_text", "label": "Seleccionar Columnas", "value": ["Nombre", "RUT", "Curso", "B", "M", "O", "Puntaje", "Rend", "SIMCE", "Nota", "Logro"], "config": {"id": "select_columns", "label": "Seleccionar Columnas", "type": "list_text", "limit": 0}}, {"id": "rename_columns", "type": "list_pair", "label": "Renombrar Columnas", "value": [{"key": "B", "val": "Buenas"}, {"key": "M", "val": "Malas"}, {"key": "O", "val": "Omitidas"}], "config": {"id": "rename_columns", "label": "Renombrar Columnas", "type": "list_pair", "limit": 0, "fields": ["Original", "Final"]}}, {"id": "enrich_data", "type": "list_pair", "label": "Enriquecer Data", "value": [{"key": "Año", "val": "2025"}, {"key": "Asignatura", "val": "Lenguaje"}, {"key": "Mes", "val": "Noviembre"}, {"key": "N Prueba", "val": "5"}], "config": {"id": "enrich_data", "label": "Enriquecer Data", "type": "list_pair", "limit": 0, "fields": ["Columna", "Valor"]}}]}</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
           <t>2026-02-13 11:50:57</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>template001.json</t>
         </is>
       </c>
     </row>
@@ -525,18 +509,16 @@
           <t>ETL Archivo</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"variables_documento": {"leftimage": "", "rightimage": "", "centerheaderone": "", "centerheadertwo": "", "centerheaderthree": "", "leftfooter": "", "rightfooter": "", "documenttitle": "", "schoolname": "", "theauthor": ""}, "secciones_fijas": [], "secciones_dinamicas": [], "etlParams": [{"id": "header_row", "type": "text", "label": "Fila Encabezado", "value": "55", "config": {"id": "header_row", "label": "Fila Encabezado", "type": "text", "limit": 1}}, {"id": "select_columns", "type": "list_text", "label": "Seleccionar Columnas", "value": ["Pregunta", "Cant.", "Cant..1", "Cant..2", "Cant..3", "Cant..4", "Correcta", "Distractor"], "config": {"id": "select_columns", "label": "Seleccionar Columnas", "type": "list_text", "limit": 0}}, {"id": "rename_columns", "type": "list_pair", "label": "Renombrar Columnas", "value": [{"key": "Cant.", "val": "A"}, {"key": "Cant..1", "val": "B"}, {"key": "Cant..2", "val": "C"}, {"key": "Cant..3", "val": "D"}, {"key": "Cant..4", "val": "E"}], "config": {"id": "rename_columns", "label": "Renombrar Columnas", "type": "list_pair", "limit": 0, "fields": ["Original", "Final"]}}, {"id": "enrich_data", "type": "list_pair", "label": "Enriquecer Data", "value": [{"key": "Año", "val": "2025"}, {"key": "Asignatura", "val": "Lenguaje"}, {"key": "Mes", "val": "Noviembre"}, {"key": "N Prueba", "val": "5"}, {"key": "Curso", "val": "", "user_input": true}], "config": {"id": "enrich_data", "label": "Enriquecer Data", "type": "list_pair", "limit": 0, "fields": ["Columna", "Valor"]}}]}</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"variables_documento": {"leftimage": "", "rightimage": "", "centerheaderone": "", "centerheadertwo": "", "centerheaderthree": "", "leftfooter": "", "rightfooter": "", "documenttitle": "", "schoolname": "", "theauthor": ""}, "secciones_fijas": [], "secciones_dinamicas": [], "etlParams": [{"id": "header_row", "type": "text", "label": "Fila Encabezado", "value": "55", "config": {"id": "header_row", "label": "Fila Encabezado", "type": "text", "limit": 1}}, {"id": "select_columns", "type": "list_text", "label": "Seleccionar Columnas", "value": ["Pregunta", "Cant.", "Cant..1", "Cant..2", "Cant..3", "Cant..4", "Correcta", "Distractor"], "config": {"id": "select_columns", "label": "Seleccionar Columnas", "type": "list_text", "limit": 0}}, {"id": "rename_columns", "type": "list_pair", "label": "Renombrar Columnas", "value": [{"key": "Cant.", "val": "A"}, {"key": "Cant..1", "val": "B"}, {"key": "Cant..2", "val": "C"}, {"key": "Cant..3", "val": "D"}, {"key": "Cant..4", "val": "E"}], "config": {"id": "rename_columns", "label": "Renombrar Columnas", "type": "list_pair", "limit": 0, "fields": ["Original", "Final"]}}, {"id": "enrich_data", "type": "list_pair", "label": "Enriquecer Data", "value": [{"key": "Año", "val": "2025"}, {"key": "Asignatura", "val": "Lenguaje"}, {"key": "Mes", "val": "Noviembre"}, {"key": "N Prueba", "val": "5"}, {"key": "Curso", "val": "", "user_input": true}], "config": {"id": "enrich_data", "label": "Enriquecer Data", "type": "list_pair", "limit": 0, "fields": ["Columna", "Valor"]}}]}</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
           <t>2026-02-28 18:22:05</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -557,18 +539,16 @@
           <t>ETL Archivo</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"etlParams": [{"id": "header_row", "type": "text", "label": "Fila Encabezado", "value": "0"}, {"id": "select_columns", "type": "list_text", "label": "Seleccionar Columnas", "value": ["N°", "Habilidad"]}]}</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{"etlParams": [{"id": "header_row", "type": "text", "label": "Fila Encabezado", "value": "0"}, {"id": "select_columns", "type": "list_text", "label": "Seleccionar Columnas", "value": ["N°", "Habilidad"]}]}</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-03-03T21:04:11.809804</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>2026-03-03 21:04:11</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -589,18 +569,16 @@
           <t>Tablas</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"metadata": {"id": "simce_lenguaje_tablas", "title": "Tablas SIMCE Lenguaje", "evaluation": "simce_lenguaje"}, "tables_list": [{"id": "resumen_logro_curso", "title": "Resumen Logro por Curso", "category": "resumen", "type": "resumen_estadistico_basico", "input_key": "df_estudiantes_prueba", "output_filename": "resumen_logro_por_curso.xlsx", "params": {"columna": "Rend", "formato": "percent", "agrupar_por": "Curso"}}, {"id": "resumen_simce_curso", "title": "Resumen SIMCE por Curso", "category": "resumen", "type": "resumen_estadistico_basico", "input_key": "df_estudiantes_prueba", "output_filename": "resumen_simce_por_curso.xlsx", "params": {"columna": "SIMCE", "formato": "number", "agrupar_por": "Curso"}}, {"id": "estadistica_por_pregunta", "title": "Estadística por Pregunta", "category": "resumen", "type": "crear_tabla_estadistica_por_pregunta", "input_key": "df_preguntas", "output_filename": "reporte_preguntas.xlsx", "params": {"parametros": {}}}, {"id": "logro_por_alumno", "title": "Logro por Alumno", "category": "detalle_curso", "type": "tabla_logro_por_alumno", "input_key": "df_estudiantes", "output_filename": "tabla_logro_por_alumno_{val}.xlsx", "iterate_by": "Curso", "params": {"parametros": {}, "sort_by": "Rend"}}, {"id": "logro_por_pregunta", "title": "Logro por Pregunta", "category": "detalle_curso", "type": "tabla_logro_por_pregunta", "input_key": "df_preguntas", "output_filename": "tabla_logro_por_pregunta_{val}.xlsx", "iterate_by": "Curso", "iterate_param": "valor_agrupacion", "params": {"agrupar_por": "Curso"}}]}</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{"metadata": {"id": "simce_lenguaje_tablas", "title": "Tablas SIMCE Lenguaje", "evaluation": "simce_lenguaje"}, "tables_list": [{"id": "resumen_logro_curso", "title": "Resumen Logro por Curso", "category": "resumen", "type": "resumen_estadistico_basico", "input_key": "df_estudiantes_prueba", "output_filename": "resumen_logro_por_curso.xlsx", "params": {"columna": "Rend", "formato": "percent", "agrupar_por": "Curso"}}, {"id": "resumen_simce_curso", "title": "Resumen SIMCE por Curso", "category": "resumen", "type": "resumen_estadistico_basico", "input_key": "df_estudiantes_prueba", "output_filename": "resumen_simce_por_curso.xlsx", "params": {"columna": "SIMCE", "formato": "number", "agrupar_por": "Curso"}}, {"id": "estadistica_por_pregunta", "title": "Estadística por Pregunta", "category": "resumen", "type": "crear_tabla_estadistica_por_pregunta", "input_key": "df_preguntas", "output_filename": "reporte_preguntas.xlsx", "params": {"parametros": {}}}, {"id": "logro_por_alumno", "title": "Logro por Alumno", "category": "detalle_curso", "type": "tabla_logro_por_alumno", "input_key": "df_estudiantes", "output_filename": "tabla_logro_por_alumno_{val}.xlsx", "iterate_by": "Curso", "params": {"parametros": {}, "sort_by": "Rend"}}, {"id": "logro_por_pregunta", "title": "Logro por Pregunta", "category": "detalle_curso", "type": "tabla_logro_por_pregunta", "input_key": "df_preguntas", "output_filename": "tabla_logro_por_pregunta_{val}.xlsx", "iterate_by": "Curso", "iterate_param": "valor_agrupacion", "params": {"agrupar_por": "Curso"}}]}</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
           <t>2026-03-05 18:21:07</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -621,14 +599,16 @@
           <t>Gráficos</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"metadata": {"id": "simce_lenguaje_graficos", "title": "Gráficos SIMCE Lenguaje", "evaluation": "simce_lenguaje"}, "charts_schema": [{"id": "rendimiento_promedio_curso", "title": "Rendimiento Promedio por Curso", "category": "resumen", "type": "grafico_barras_promedio_por", "input_key": "df_estudiantes_prueba", "output_filename": "rendimiento_promedio_por_curso.png", "params": {"columna_valor": "Rend", "agrupar_por": "Curso", "titulo": "Rendimiento Promedio por Curso", "ylabel": "Rendimiento (%)"}}, {"id": "distribucion_simce_curso", "title": "Distribución de Puntaje SIMCE por Curso", "category": "resumen", "type": "boxplot_valor_por_curso", "input_key": "df_estudiantes_prueba", "output_filename": "distribucion_puntaje_simce_por_curso.png", "params": {"columna_valor": "SIMCE", "agrupar_por": "Curso", "titulo_grafico": "Distribución de Puntaje SIMCE por Curso", "ylabel": "Puntaje SIMCE", "formato": "number"}}, {"id": "alumnos_por_nivel_curso", "title": "Alumnos por Nivel de Logro y Curso", "category": "resumen", "type": "alumnos_por_nivel_cualitativo", "input_key": "df_estudiantes_prueba", "output_filename": "alumnos_por_nivel.png", "params": {"columna_nivel": "Logro", "agrupar_por": "Curso", "titulo_grafico": "Cantidad de Alumnos por Nivel de Logro y Curso", "titulo_leyenda": "Nivel de Logro", "ylabel": "Cantidad de Alumnos"}}, {"id": "evolucion_logro_mes", "title": "Evolución del Logro Promedio por Curso y Mes", "category": "evolucion", "type": "valor_promedio_agrupado_por", "input_key": "df_estudiantes", "output_filename": "evolucion_logro_promedio_por_curso_y_mes.png", "params": {"columna_valor": "Rend", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Mes", "titulo_grafico": "Evolución del Logro Promedio por Curso y Mes", "titulo_leyenda": "Mes", "y_lims": [0, 1], "formato": "percent"}}, {"id": "evolucion_simce_mes", "title": "Evolución del SIMCE Promedio por Curso y Mes", "category": "evolucion", "type": "valor_promedio_agrupado_por", "input_key": "df_estudiantes", "output_filename": "evolucion_simce_promedio_por_curso_y_mes.png", "params": {"columna_valor": "SIMCE", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Mes", "titulo_grafico": "Evolución del SIMCE Promedio por Curso y Mes", "titulo_leyenda": "Mes", "formato": "number"}}, {"id": "evolucion_alumnos_nivel_mes", "title": "Evolución de Alumnos por Nivel y Mes", "category": "evolucion", "type": "alumnos_por_nivel_curso_y_mes", "input_key": "df_estudiantes", "output_filename": "evolucion_alumnos_por_nivel.png", "params": {"columna_nivel": "Logro", "titulo_grafico": "", "titulo_leyenda": "Nivel de Logro", "ylabel": "Cantidad de Alumnos"}}, {"id": "logro_por_habilidad", "title": "Logro Promedio por Habilidad", "category": "preguntas", "type": "valor_promedio_agrupado_por", "input_key": "df_preguntas", "output_filename": "logro_promedio_por_habilidad.png", "params": {"columna_valor": "Logro", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Habilidad", "titulo_grafico": "Logro Promedio por Habilidad", "titulo_leyenda": "Habilidad", "formato": "percent"}}, {"id": "logro_por_eje", "title": "Logro Promedio por Eje Temático", "category": "preguntas", "type": "valor_promedio_agrupado_por", "input_key": "df_preguntas", "output_filename": "logro_promedio_por_eje.png", "params": {"columna_valor": "Logro", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Eje temático", "titulo_grafico": "Logro Promedio por Eje Temático", "titulo_leyenda": "Eje Temático", "formato": "percent"}}]}</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{"metadata": {"id": "simce_lenguaje_graficos", "title": "Gráficos SIMCE Lenguaje", "evaluation": "simce_lenguaje"}, "charts_schema": [{"id": "rendimiento_promedio_curso", "title": "Rendimiento Promedio por Curso", "category": "resumen", "type": "grafico_barras_promedio_por", "input_key": "df_estudiantes_prueba", "output_filename": "rendimiento_promedio_por_curso.png", "params": {"columna_valor": "Rend", "agrupar_por": "Curso", "titulo": "Rendimiento Promedio por Curso", "ylabel": "Rendimiento (%)"}}, {"id": "distribucion_simce_curso", "title": "Distribución de Puntaje SIMCE por Curso", "category": "resumen", "type": "boxplot_valor_por_curso", "input_key": "df_estudiantes_prueba", "output_filename": "distribucion_puntaje_simce_por_curso.png", "params": {"columna_valor": "SIMCE", "agrupar_por": "Curso", "titulo_grafico": "Distribución de Puntaje SIMCE por Curso", "ylabel": "Puntaje SIMCE", "formato": "number"}}, {"id": "alumnos_por_nivel_curso", "title": "Alumnos por Nivel de Logro y Curso", "category": "resumen", "type": "alumnos_por_nivel_cualitativo", "input_key": "df_estudiantes_prueba", "output_filename": "alumnos_por_nivel.png", "params": {"columna_nivel": "Logro", "agrupar_por": "Curso", "titulo_grafico": "Cantidad de Alumnos por Nivel de Logro y Curso", "titulo_leyenda": "Nivel de Logro", "ylabel": "Cantidad de Alumnos"}}, {"id": "evolucion_logro_mes", "title": "Evolución del Logro Promedio por Curso y Mes", "category": "evolucion", "type": "valor_promedio_agrupado_por", "input_key": "df_estudiantes", "output_filename": "evolucion_logro_promedio_por_curso_y_mes.png", "params": {"columna_valor": "Rend", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Mes", "titulo_grafico": "Evolución del Logro Promedio por Curso y Mes", "titulo_leyenda": "Mes", "y_lims": [0, 1], "formato": "percent"}}, {"id": "evolucion_simce_mes", "title": "Evolución del SIMCE Promedio por Curso y Mes", "category": "evolucion", "type": "valor_promedio_agrupado_por", "input_key": "df_estudiantes", "output_filename": "evolucion_simce_promedio_por_curso_y_mes.png", "params": {"columna_valor": "SIMCE", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Mes", "titulo_grafico": "Evolución del SIMCE Promedio por Curso y Mes", "titulo_leyenda": "Mes", "formato": "number"}}, {"id": "evolucion_alumnos_nivel_mes", "title": "Evolución de Alumnos por Nivel y Mes", "category": "evolucion", "type": "alumnos_por_nivel_curso_y_mes", "input_key": "df_estudiantes", "output_filename": "evolucion_alumnos_por_nivel.png", "params": {"columna_nivel": "Logro", "titulo_grafico": "", "titulo_leyenda": "Nivel de Logro", "ylabel": "Cantidad de Alumnos"}}, {"id": "logro_por_habilidad", "title": "Logro Promedio por Habilidad", "category": "preguntas", "type": "valor_promedio_agrupado_por", "input_key": "df_preguntas", "output_filename": "logro_promedio_por_habilidad.png", "params": {"columna_valor": "Logro", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Habilidad", "titulo_grafico": "Logro Promedio por Habilidad", "titulo_leyenda": "Habilidad", "formato": "percent"}}, {"id": "logro_por_eje", "title": "Logro Promedio por Eje Temático", "category": "preguntas", "type": "valor_promedio_agrupado_por", "input_key": "df_preguntas", "output_filename": "logro_promedio_por_eje.png", "params": {"columna_valor": "Logro", "agrupar_principal_por": "Curso", "agrupar_secundario_por": "Eje temático", "titulo_grafico": "Logro Promedio por Eje Temático", "titulo_leyenda": "Eje Temático", "formato": "percent"}}]}</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+          <t>2026-03-06 08:54:42</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>